<commit_message>
fix: revisions and comments in office
</commit_message>
<xml_diff>
--- a/public/test.xlsx
+++ b/public/test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="17200"/>
+    <workbookView windowHeight="15520"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="4">
   <si>
     <t>test_</t>
+  </si>
+  <si>
+    <t>测试自定义字体</t>
+  </si>
+  <si>
+    <t>other</t>
   </si>
   <si>
     <t>dsadsa</t>
@@ -46,13 +52,19 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="仿宋_GB2312"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -512,64 +524,64 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -578,10 +590,10 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -590,10 +602,10 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -602,10 +614,10 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -614,10 +626,10 @@
     <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -626,10 +638,10 @@
     <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -638,12 +650,15 @@
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -910,7 +925,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{37CB6C28-DD74-B216-DABC-19698F6B68DE}">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{BE38E8D2-B6CD-1A8D-0F81-266AAC4B50EF}">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -919,7 +934,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{C46DCFE5-EE92-DA7C-DABC-1969762CE584}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{4428D59F-379A-A0F4-0F81-266A6AD7CBD5}">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -938,13 +953,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1191,163 +1199,173 @@
   <dimension ref="A1:Q27"/>
   <sheetFormatPr defaultColWidth="9.23214285714286" defaultRowHeight="16.8"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="11:12">
+    <row r="3" spans="1:17">
+      <c r="C3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="K5" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="10:15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="J6" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="O8" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P8" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="O9" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P9" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q9" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
       <c r="O10" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P10" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="10:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
       <c r="J11" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O11" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P11" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
       <c r="O12" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
       <c r="O13" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P13" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="11:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
       <c r="K14" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O14" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P14" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
       <c r="O15" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P15" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q15" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
       <c r="O16" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P16" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q16" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="7:17">
       <c r="O17" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P17" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q17" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="7:17">
       <c r="O18" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P18" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q18" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="7:17">
       <c r="O19" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P19" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q19" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="7:17">
@@ -1355,90 +1373,90 @@
         <v>23</v>
       </c>
       <c r="O20" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P20" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q20" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="7:17">
       <c r="O21" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P21" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q21" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="7:17">
       <c r="O22" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P22" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q22" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="7:17">
       <c r="O23" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P23" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q23" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="7:17">
       <c r="O24" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P24" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q24" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="7:17">
       <c r="O25" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P25" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q25" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="7:17">
       <c r="O26" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P26" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q26" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="15:17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="7:17">
       <c r="O27" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P27" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q27" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>